<commit_message>
add responsive for other devices
</commit_message>
<xml_diff>
--- a/src/locales/languages.xlsx
+++ b/src/locales/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/tax-calculator/src/locales/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{687E3E19-4DCD-A848-936D-0E4414AAB7C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D648FDAC-0BA0-9C46-A756-5509BAD1DA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="27320" windowHeight="14240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="150">
   <si>
     <t>Key</t>
   </si>
@@ -223,47 +223,6 @@
   </si>
   <si>
     <t>通知</t>
-  </si>
-  <si>
-    <t>home.answer.no-tax</t>
-  </si>
-  <si>
-    <t>Your taxable income is negative, no need to pay tax</t>
-  </si>
-  <si>
-    <t>Thu nhập tính thuế của bạn &lt; 0, chưa đến mức phải nộp thuế</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="13"/>
-        <color rgb="FF000000"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">課税所得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="13"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t>&lt; 0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="13"/>
-        <color rgb="FF000000"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>、まだ課税対象外です</t>
-    </r>
   </si>
   <si>
     <t>home.answer-net.row-1</t>
@@ -791,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D488"/>
+  <dimension ref="A1:D487"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.5" style="1" customWidth="1"/>
@@ -1052,7 +1011,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="36" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>66</v>
       </c>
@@ -1071,38 +1030,38 @@
         <v>70</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>72</v>
+        <v>138</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>73</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>143</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>77</v>
+        <v>136</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>144</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>76</v>
@@ -1110,44 +1069,44 @@
     </row>
     <row r="23" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>140</v>
+        <v>77</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>79</v>
+        <v>141</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>71</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="20" x14ac:dyDescent="0.2">
@@ -1292,58 +1251,58 @@
     </row>
     <row r="36" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>125</v>
+        <v>142</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="20" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>137</v>
+        <v>123</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>125</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="20" x14ac:dyDescent="0.2">
@@ -1365,28 +1324,20 @@
         <v>131</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>132</v>
+        <v>96</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="20" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
     </row>
     <row r="43" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="3"/>
@@ -1833,7 +1784,7 @@
       <c r="D116" s="4"/>
     </row>
     <row r="117" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="3"/>
+      <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
       <c r="D117" s="4"/>
@@ -1845,7 +1796,7 @@
       <c r="D118" s="4"/>
     </row>
     <row r="119" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A119" s="4"/>
+      <c r="A119" s="3"/>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
       <c r="D119" s="4"/>
@@ -2248,8 +2199,8 @@
     </row>
     <row r="186" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A186" s="3"/>
-      <c r="B186" s="4"/>
-      <c r="C186" s="4"/>
+      <c r="B186" s="6"/>
+      <c r="C186" s="6"/>
       <c r="D186" s="4"/>
     </row>
     <row r="187" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2278,8 +2229,8 @@
     </row>
     <row r="191" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A191" s="3"/>
-      <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
+      <c r="B191" s="4"/>
+      <c r="C191" s="4"/>
       <c r="D191" s="4"/>
     </row>
     <row r="192" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2326,8 +2277,8 @@
     </row>
     <row r="199" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A199" s="3"/>
-      <c r="B199" s="4"/>
-      <c r="C199" s="4"/>
+      <c r="B199" s="6"/>
+      <c r="C199" s="6"/>
       <c r="D199" s="4"/>
     </row>
     <row r="200" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2356,8 +2307,8 @@
     </row>
     <row r="204" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A204" s="3"/>
-      <c r="B204" s="6"/>
-      <c r="C204" s="6"/>
+      <c r="B204" s="4"/>
+      <c r="C204" s="4"/>
       <c r="D204" s="4"/>
     </row>
     <row r="205" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -3190,13 +3141,13 @@
     </row>
     <row r="343" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A343" s="3"/>
-      <c r="B343" s="4"/>
+      <c r="B343" s="3"/>
       <c r="C343" s="4"/>
       <c r="D343" s="4"/>
     </row>
     <row r="344" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A344" s="3"/>
-      <c r="B344" s="3"/>
+      <c r="B344" s="4"/>
       <c r="C344" s="4"/>
       <c r="D344" s="4"/>
     </row>
@@ -3400,7 +3351,7 @@
     </row>
     <row r="378" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A378" s="3"/>
-      <c r="B378" s="4"/>
+      <c r="B378" s="3"/>
       <c r="C378" s="4"/>
       <c r="D378" s="4"/>
     </row>
@@ -3412,7 +3363,7 @@
     </row>
     <row r="380" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A380" s="3"/>
-      <c r="B380" s="3"/>
+      <c r="B380" s="4"/>
       <c r="C380" s="4"/>
       <c r="D380" s="4"/>
     </row>
@@ -3850,15 +3801,15 @@
     </row>
     <row r="453" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A453" s="3"/>
-      <c r="B453" s="4"/>
-      <c r="C453" s="4"/>
-      <c r="D453" s="4"/>
+      <c r="B453" s="3"/>
+      <c r="C453" s="3"/>
+      <c r="D453" s="3"/>
     </row>
     <row r="454" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A454" s="3"/>
-      <c r="B454" s="3"/>
-      <c r="C454" s="3"/>
-      <c r="D454" s="3"/>
+      <c r="B454" s="4"/>
+      <c r="C454" s="4"/>
+      <c r="D454" s="4"/>
     </row>
     <row r="455" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A455" s="3"/>
@@ -3928,9 +3879,9 @@
     </row>
     <row r="466" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A466" s="3"/>
-      <c r="B466" s="4"/>
-      <c r="C466" s="4"/>
-      <c r="D466" s="4"/>
+      <c r="B466" s="3"/>
+      <c r="C466" s="3"/>
+      <c r="D466" s="3"/>
     </row>
     <row r="467" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A467" s="3"/>
@@ -3958,9 +3909,9 @@
     </row>
     <row r="471" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A471" s="3"/>
-      <c r="B471" s="3"/>
-      <c r="C471" s="3"/>
-      <c r="D471" s="3"/>
+      <c r="B471" s="4"/>
+      <c r="C471" s="4"/>
+      <c r="D471" s="4"/>
     </row>
     <row r="472" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A472" s="3"/>
@@ -4048,21 +3999,15 @@
     </row>
     <row r="486" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A486" s="3"/>
-      <c r="B486" s="4"/>
-      <c r="C486" s="4"/>
-      <c r="D486" s="4"/>
+      <c r="B486" s="3"/>
+      <c r="C486" s="3"/>
+      <c r="D486" s="3"/>
     </row>
     <row r="487" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A487" s="3"/>
       <c r="B487" s="3"/>
       <c r="C487" s="3"/>
       <c r="D487" s="3"/>
-    </row>
-    <row r="488" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A488" s="3"/>
-      <c r="B488" s="3"/>
-      <c r="C488" s="3"/>
-      <c r="D488" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
add chinese and set vietnamese as default
</commit_message>
<xml_diff>
--- a/src/locales/languages.xlsx
+++ b/src/locales/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/tax-calculator/src/locales/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EA5C79-E14B-0942-B775-3B3F965ABFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794FC8B0-31AE-DA4C-9552-2F6FB0F9010E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="27320" windowHeight="14240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="225">
   <si>
     <t>Key</t>
   </si>
@@ -586,13 +586,127 @@
   </si>
   <si>
     <t>급여 및 세금 세부 정보</t>
+  </si>
+  <si>
+    <t>Chinese</t>
+  </si>
+  <si>
+    <t>必填</t>
+  </si>
+  <si>
+    <t>個人所得稅計算器</t>
+  </si>
+  <si>
+    <t>收入</t>
+  </si>
+  <si>
+    <t>輸入收入</t>
+  </si>
+  <si>
+    <t>受扶養人</t>
+  </si>
+  <si>
+    <t>輸入受扶養人</t>
+  </si>
+  <si>
+    <t>繳費等級</t>
+  </si>
+  <si>
+    <t>以正式工資計算</t>
+  </si>
+  <si>
+    <t>其他</t>
+  </si>
+  <si>
+    <t>繳費金額</t>
+  </si>
+  <si>
+    <t>至少 {0}₫</t>
+  </si>
+  <si>
+    <t>目標工資類型</t>
+  </si>
+  <si>
+    <t>淨收入</t>
+  </si>
+  <si>
+    <t>總收入</t>
+  </si>
+  <si>
+    <t>計算至 {0}</t>
+  </si>
+  <si>
+    <t>薪資和稅務詳情</t>
+  </si>
+  <si>
+    <t>總收入為 {0}₫</t>
+  </si>
+  <si>
+    <t>已繳保險費為 {0}₫</t>
+  </si>
+  <si>
+    <t>稅前收入為 {0}₫</t>
+  </si>
+  <si>
+    <t>應稅所得為 {0}₫</t>
+  </si>
+  <si>
+    <t>稅額為 {0}₫</t>
+  </si>
+  <si>
+    <t>淨收入為 {0}₫</t>
+  </si>
+  <si>
+    <t>語言</t>
+  </si>
+  <si>
+    <t>深色模式</t>
+  </si>
+  <si>
+    <t>關閉</t>
+  </si>
+  <si>
+    <t>個人扣除額</t>
+  </si>
+  <si>
+    <t>受扶養人扣除額</t>
+  </si>
+  <si>
+    <t>保險費率</t>
+  </si>
+  <si>
+    <t>最低保險基數</t>
+  </si>
+  <si>
+    <t>個人所得稅政策</t>
+  </si>
+  <si>
+    <t>04/2007/QH12 號 法律</t>
+  </si>
+  <si>
+    <t>第 954/2020/UBTVQH14 號決議</t>
+  </si>
+  <si>
+    <t>第 110/2025/UBTVQH15 號決議</t>
+  </si>
+  <si>
+    <t>稅收政策詳情</t>
+  </si>
+  <si>
+    <t>稅級</t>
+  </si>
+  <si>
+    <t>稅階</t>
+  </si>
+  <si>
+    <t>稅率</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -627,6 +741,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -648,7 +768,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -668,6 +788,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -861,7 +982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E486"/>
+  <dimension ref="A1:F486"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.5" style="1" customWidth="1"/>
@@ -869,9 +990,10 @@
     <col min="3" max="3" width="42.1640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="40.1640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="30" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="36.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -887,8 +1009,11 @@
       <c r="E1" s="4" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F1" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -904,8 +1029,11 @@
       <c r="E2" s="4" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F2" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -921,8 +1049,11 @@
       <c r="E3" s="4" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F3" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -938,8 +1069,11 @@
       <c r="E4" s="4" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F4" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
@@ -955,8 +1089,11 @@
       <c r="E5" s="4" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F5" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
@@ -972,8 +1109,11 @@
       <c r="E6" s="4" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F6" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -989,8 +1129,11 @@
       <c r="E7" s="4" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F7" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>28</v>
       </c>
@@ -1006,8 +1149,11 @@
       <c r="E8" s="4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F8" s="7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1023,8 +1169,11 @@
       <c r="E9" s="4" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F9" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>36</v>
       </c>
@@ -1040,8 +1189,11 @@
       <c r="E10" s="4" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F10" s="7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>40</v>
       </c>
@@ -1057,8 +1209,11 @@
       <c r="E11" s="4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F11" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>42</v>
       </c>
@@ -1074,8 +1229,11 @@
       <c r="E12" s="4" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F12" s="7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>46</v>
       </c>
@@ -1091,8 +1249,11 @@
       <c r="E13" s="4" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F13" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>50</v>
       </c>
@@ -1108,8 +1269,11 @@
       <c r="E14" s="4" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F14" s="7" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>52</v>
       </c>
@@ -1125,8 +1289,11 @@
       <c r="E15" s="4" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F15" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>54</v>
       </c>
@@ -1142,8 +1309,11 @@
       <c r="E16" s="4" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F16" s="7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>58</v>
       </c>
@@ -1159,8 +1329,11 @@
       <c r="E17" s="4" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F17" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>110</v>
       </c>
@@ -1176,8 +1349,11 @@
       <c r="E18" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F18" s="7" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>111</v>
       </c>
@@ -1193,8 +1369,11 @@
       <c r="E19" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F19" s="7" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>112</v>
       </c>
@@ -1210,8 +1389,11 @@
       <c r="E20" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F20" s="7" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>113</v>
       </c>
@@ -1227,8 +1409,11 @@
       <c r="E21" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F21" s="7" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>114</v>
       </c>
@@ -1244,8 +1429,11 @@
       <c r="E22" s="4" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F22" s="7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>115</v>
       </c>
@@ -1261,8 +1449,11 @@
       <c r="E23" s="4" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F23" s="7" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>62</v>
       </c>
@@ -1278,8 +1469,11 @@
       <c r="E24" s="4" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F24" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>66</v>
       </c>
@@ -1295,8 +1489,11 @@
       <c r="E25" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F25" s="7" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>70</v>
       </c>
@@ -1312,8 +1509,11 @@
       <c r="E26" s="4" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F26" s="7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>74</v>
       </c>
@@ -1329,8 +1529,11 @@
       <c r="E27" s="4" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F27" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>78</v>
       </c>
@@ -1346,8 +1549,11 @@
       <c r="E28" s="4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F28" s="7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>82</v>
       </c>
@@ -1363,8 +1569,11 @@
       <c r="E29" s="4" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F29" s="7" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>86</v>
       </c>
@@ -1380,8 +1589,11 @@
       <c r="E30" s="4" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F30" s="7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>90</v>
       </c>
@@ -1397,8 +1609,11 @@
       <c r="E31" s="4" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F31" s="7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>159</v>
       </c>
@@ -1414,8 +1629,11 @@
       <c r="E32" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F32" s="7" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>162</v>
       </c>
@@ -1431,8 +1649,11 @@
       <c r="E33" s="4" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F33" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>163</v>
       </c>
@@ -1448,8 +1669,11 @@
       <c r="E34" s="4" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F34" s="7" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>164</v>
       </c>
@@ -1465,8 +1689,11 @@
       <c r="E35" s="4" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F35" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>178</v>
       </c>
@@ -1482,8 +1709,11 @@
       <c r="E36" s="4" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F36" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>155</v>
       </c>
@@ -1499,8 +1729,11 @@
       <c r="E37" s="4" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F37" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>153</v>
       </c>
@@ -1516,8 +1749,11 @@
       <c r="E38" s="4" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F38" s="7" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>154</v>
       </c>
@@ -1533,8 +1769,11 @@
       <c r="E39" s="4" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="20" x14ac:dyDescent="0.2">
+      <c r="F39" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>94</v>
       </c>
@@ -1550,50 +1789,53 @@
       <c r="E40" s="4" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F40" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>

</xml_diff>